<commit_message>
ajustando códigos e templates
</commit_message>
<xml_diff>
--- a/Templates/XLS-MATRIZ.xlsx
+++ b/Templates/XLS-MATRIZ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pablo\DDVMigracao\DDVMigracao\bin\Debug\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DDVRefatorado\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{25CF6132-F9B0-4D74-970A-064C9F545F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C73AB0ED-EDDF-47A4-9812-1897F5174B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{2E54BBDE-98B4-4833-95CB-76D96253B1CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{5B1D5280-5086-4CF9-819B-9159FD3094D5}"/>
   </bookViews>
   <sheets>
     <sheet name="TOTINDICE" sheetId="1" r:id="rId1"/>
@@ -1573,7 +1573,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B63178C-60F3-4C94-BF24-4413C5A02CED}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD3A034F-10B9-46C3-B15B-F5E057419407}">
   <dimension ref="A1:L678"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="15"/>
   <cols>
@@ -9736,7 +9736,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17072359-3A27-4F20-9895-6073ECD0F2B5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E450C8E5-A57B-4326-B7CB-CE755C602F70}">
   <dimension ref="A3:N28"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="16.5"/>
   <cols>

</xml_diff>

<commit_message>
Remoção das colunas inutilizadas do excel e otimização do app.py
</commit_message>
<xml_diff>
--- a/Templates/XLS-MATRIZ.xlsx
+++ b/Templates/XLS-MATRIZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cloudprodamazhotmail-my.sharepoint.com/personal/pedroferrari_prodam_sp_gov_br/Documents/Área de Trabalho/ddv/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="8_{25CF6132-F9B0-4D74-970A-064C9F545F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9CA65F1-92ED-4EEE-856D-8E7EC2FDE97D}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="8_{25CF6132-F9B0-4D74-970A-064C9F545F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AF11806-5CA3-4F86-BA2D-314D33B52758}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{2E54BBDE-98B4-4833-95CB-76D96253B1CE}"/>
   </bookViews>
@@ -613,7 +613,7 @@
     <numFmt numFmtId="169" formatCode="0.000000%"/>
     <numFmt numFmtId="170" formatCode="&quot;R$&quot;\ 0.00"/>
     <numFmt numFmtId="171" formatCode="&quot;R$&quot;\ #,#00.00"/>
-    <numFmt numFmtId="173" formatCode="\R\$#,#00.00"/>
+    <numFmt numFmtId="172" formatCode="\R\$#,#00.00"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -983,7 +983,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1101,14 +1101,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="173" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -9688,8 +9688,8 @@
       <c r="B7" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="89"/>
-      <c r="D7" s="90"/>
+      <c r="C7" s="90"/>
+      <c r="D7" s="91"/>
       <c r="E7" s="12" t="s">
         <v>19</v>
       </c>
@@ -9856,7 +9856,7 @@
       <c r="A23" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="91" t="e">
+      <c r="D23" s="89" t="e">
         <f>C20-D20-E20</f>
         <v>#N/A</v>
       </c>
@@ -9865,13 +9865,13 @@
       <c r="A24" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="91"/>
+      <c r="D24" s="89"/>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="91">
+      <c r="D25" s="89">
         <f>D20+F20+G20</f>
         <v>0</v>
       </c>
@@ -9880,7 +9880,7 @@
       <c r="A26" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D26" s="91">
+      <c r="D26" s="89">
         <f>E20</f>
         <v>0</v>
       </c>
@@ -9889,7 +9889,7 @@
       <c r="A27" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D27" s="91" t="e">
+      <c r="D27" s="89" t="e">
         <f>SUM(D23:D26)</f>
         <v>#N/A</v>
       </c>

</xml_diff>